<commit_message>
Update Excel data, swap combo logo, fix Active Targets height with ResizeObserver
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/NuSilq/Silq-NuSil ongoing projects Offline.xlsx
+++ b/NuSilq/Silq-NuSil ongoing projects Offline.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7ef4039dce562a81/Desktop/Webdev/NuSilq/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brianmcverry/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="44" documentId="8_{0C68F5CF-D9AC-402E-8D89-54912A076CF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DD22817-00BF-4151-91C3-E29600CE46E8}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A80F975F-EEB6-314D-94BA-97FB57470EE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="100680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3890AACB-A675-4B39-BB5E-5805C6E09923}"/>
+    <workbookView xWindow="1660" yWindow="1680" windowWidth="26520" windowHeight="15440" activeTab="2" xr2:uid="{3890AACB-A675-4B39-BB5E-5805C6E09923}"/>
   </bookViews>
   <sheets>
     <sheet name="Ongoing Projects" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="149">
   <si>
     <t>Company Name</t>
   </si>
@@ -295,6 +294,9 @@
     <t>Notes</t>
   </si>
   <si>
+    <t>Challenge</t>
+  </si>
+  <si>
     <t>Device Details</t>
   </si>
   <si>
@@ -307,6 +309,9 @@
     <t>Baerveldt nonvalved Implant J&amp;J</t>
   </si>
   <si>
+    <t>Occlusion, infection, bleeding, hypontony</t>
+  </si>
+  <si>
     <t>Silicone device includes holes to allow fibrous tissue growth</t>
   </si>
   <si>
@@ -346,9 +351,6 @@
     <t>Aspero Medical</t>
   </si>
   <si>
-    <t xml:space="preserve">They have not made a decision yet.  Need to follow up. </t>
-  </si>
-  <si>
     <t>Hydrocephalous</t>
   </si>
   <si>
@@ -391,24 +393,15 @@
     <t>Meeting at MD&amp;M.  Callon 2/12/26</t>
   </si>
   <si>
+    <t>Fibrosis and friction</t>
+  </si>
+  <si>
     <t>Nexsilis</t>
   </si>
   <si>
-    <t>Medicone</t>
-  </si>
-  <si>
-    <t>FAJ</t>
-  </si>
-  <si>
-    <t>IBEG</t>
-  </si>
-  <si>
     <t>Gabisa</t>
   </si>
   <si>
-    <t>Faga Medical</t>
-  </si>
-  <si>
     <t>Breastimplant with PU foam setcion.  May want echogenic silicone</t>
   </si>
   <si>
@@ -461,13 +454,43 @@
   </si>
   <si>
     <t>Electrochemical analysis, performance testing starting Q3</t>
+  </si>
+  <si>
+    <t>Osstem Implant (Korea)</t>
+  </si>
+  <si>
+    <t>BS Research (Korea)</t>
+  </si>
+  <si>
+    <t>Hans Biomed (Korea)</t>
+  </si>
+  <si>
+    <t>Medicone (Brazil)</t>
+  </si>
+  <si>
+    <t>Silimed (Brazil)</t>
+  </si>
+  <si>
+    <t>FAJ (Brazil)</t>
+  </si>
+  <si>
+    <t>IBEG (Brazil)</t>
+  </si>
+  <si>
+    <t>Faga Medical (Brazil)</t>
+  </si>
+  <si>
+    <t>Active Project</t>
+  </si>
+  <si>
+    <t>Lubiricity on inside of Endoscopic Sleeve device</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -509,6 +532,12 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FF242424"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos"/>
       <family val="2"/>
@@ -541,7 +570,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -576,6 +605,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -601,10 +633,11 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -620,10 +653,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -944,26 +973,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76AAE435-38A4-4168-BBF1-B1C51AFD5BDE}">
   <dimension ref="A1:G16"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="46" style="6" customWidth="1"/>
-    <col min="2" max="2" width="41.59765625" style="6" customWidth="1"/>
-    <col min="3" max="3" width="58.265625" style="8" customWidth="1"/>
+    <col min="2" max="2" width="41.6640625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="58.33203125" style="8" customWidth="1"/>
     <col min="4" max="4" width="24" style="6" customWidth="1"/>
-    <col min="5" max="5" width="36.73046875" style="14" customWidth="1"/>
-    <col min="6" max="6" width="42.265625" style="14" customWidth="1"/>
-    <col min="7" max="7" width="19.73046875" style="14" customWidth="1"/>
-    <col min="8" max="16384" width="9.1328125" style="14"/>
+    <col min="5" max="5" width="36.6640625" style="15" customWidth="1"/>
+    <col min="6" max="6" width="42.33203125" style="15" customWidth="1"/>
+    <col min="7" max="7" width="19.6640625" style="15" customWidth="1"/>
+    <col min="8" max="16384" width="9.1640625" style="15"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="14" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -976,35 +1005,35 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>135</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>137</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="21">
+      <c r="E2" s="23">
         <v>46182</v>
       </c>
-      <c r="F2" s="14" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="F2" s="15" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>32</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>7</v>
@@ -1016,61 +1045,61 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15.75" x14ac:dyDescent="0.35">
-      <c r="A4" s="22" t="s">
+    <row r="4" spans="1:7" ht="17" x14ac:dyDescent="0.15">
+      <c r="A4" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C4" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="E4" s="23">
+        <v>46174</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="E4" s="21">
-        <v>46174</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+    </row>
+    <row r="5" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>45</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="E5" s="21">
+        <v>131</v>
+      </c>
+      <c r="E5" s="23">
         <v>46174</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="E6" s="23">
+        <v>46174</v>
+      </c>
+      <c r="F6" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="C6" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="E6" s="21">
-        <v>46174</v>
-      </c>
-      <c r="F6" s="14" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
+    </row>
+    <row r="7" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
         <v>14</v>
       </c>
@@ -1080,14 +1109,14 @@
       <c r="C7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="15">
+      <c r="E7" s="16">
         <v>45912</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
         <v>9</v>
       </c>
@@ -1102,7 +1131,7 @@
       </c>
       <c r="F8" s="6"/>
     </row>
-    <row r="9" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -1117,7 +1146,7 @@
       </c>
       <c r="F9" s="6"/>
     </row>
-    <row r="10" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>18</v>
       </c>
@@ -1137,7 +1166,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
         <v>21</v>
       </c>
@@ -1147,14 +1176,14 @@
       <c r="D11" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="15">
+      <c r="E11" s="16">
         <v>45839</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
         <v>25</v>
       </c>
@@ -1164,12 +1193,12 @@
       <c r="C12" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="E12" s="15">
+      <c r="E12" s="16">
         <v>45839</v>
       </c>
       <c r="F12" s="6"/>
     </row>
-    <row r="13" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>28</v>
       </c>
@@ -1190,7 +1219,7 @@
       </c>
       <c r="G13" s="6"/>
     </row>
-    <row r="14" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>33</v>
       </c>
@@ -1206,7 +1235,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>36</v>
       </c>
@@ -1222,7 +1251,7 @@
       </c>
       <c r="F15" s="4"/>
     </row>
-    <row r="16" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
         <v>38</v>
       </c>
@@ -1250,29 +1279,29 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B84007B7-3687-44DF-97CF-1AF65736DFED}">
   <dimension ref="A1:E22"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.3984375" style="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="62.86328125" style="16" customWidth="1"/>
-    <col min="3" max="3" width="40.1328125" style="16" customWidth="1"/>
-    <col min="4" max="4" width="17" style="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.33203125" style="13" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="62.83203125" style="17" customWidth="1"/>
+    <col min="3" max="3" width="40.1640625" style="17" customWidth="1"/>
+    <col min="4" max="4" width="17" style="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="18" t="s">
         <v>5</v>
       </c>
       <c r="D1" s="9" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>42</v>
       </c>
@@ -1286,11 +1315,11 @@
         <v>45729</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C3" s="7"/>
       <c r="D3" s="4"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>46</v>
       </c>
@@ -1298,7 +1327,7 @@
       <c r="C4" s="7"/>
       <c r="D4" s="4"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>47</v>
       </c>
@@ -1306,7 +1335,7 @@
       <c r="C5" s="7"/>
       <c r="D5" s="4"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>48</v>
       </c>
@@ -1314,7 +1343,7 @@
       <c r="C6" s="7"/>
       <c r="D6" s="4"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>49</v>
       </c>
@@ -1322,7 +1351,7 @@
       <c r="C7" s="7"/>
       <c r="D7" s="4"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>50</v>
       </c>
@@ -1330,7 +1359,7 @@
       <c r="C8" s="7"/>
       <c r="D8" s="4"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>51</v>
       </c>
@@ -1342,7 +1371,7 @@
         <v>45590</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>53</v>
       </c>
@@ -1350,92 +1379,92 @@
       <c r="C10" s="7"/>
       <c r="D10" s="4"/>
     </row>
-    <row r="11" spans="1:4" ht="42.75" x14ac:dyDescent="0.45">
-      <c r="A11" s="12" t="s">
+    <row r="11" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+      <c r="A11" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="D11" s="19">
+      <c r="D11" s="20">
         <v>44474</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A12" s="12" t="s">
+    <row r="12" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A12" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="B12" s="16" t="s">
+      <c r="B12" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="D12" s="19">
+      <c r="D12" s="20">
         <v>44697</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A13" s="12" t="s">
+    <row r="13" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A13" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="17" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A14" s="12" t="s">
+    <row r="14" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A14" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="D14" s="19">
+      <c r="D14" s="20">
         <v>45240</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A15" s="12" t="s">
+    <row r="15" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A15" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="B15" s="16" t="s">
+      <c r="B15" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="C15" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="D15" s="19">
+      <c r="D15" s="20">
         <v>45810</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A16" s="12" t="s">
+    <row r="16" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A16" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="B16" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="C16" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="D16" s="12" t="s">
+      <c r="D16" s="13" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>72</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="19" t="s">
         <v>74</v>
       </c>
       <c r="D17" s="5">
@@ -1445,12 +1474,12 @@
         <v>74</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A18" s="12" t="s">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="13" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="38.25" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>76</v>
       </c>
@@ -1464,7 +1493,7 @@
         <v>45700</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A20" s="6" t="s">
         <v>78</v>
       </c>
@@ -1478,23 +1507,23 @@
         <v>45791</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A21" s="12" t="s">
+    <row r="21" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A21" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="B21" s="16" t="s">
+      <c r="B21" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="D21" s="19">
+      <c r="D21" s="20">
         <v>46107</v>
       </c>
     </row>
-    <row r="22" spans="1:5" s="14" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:5" s="15" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>8</v>
@@ -1510,260 +1539,309 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8C8D27E-B004-4030-B562-9BB31DA23028}">
-  <dimension ref="A1:E29"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:G29"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.86328125" customWidth="1"/>
-    <col min="2" max="2" width="37.265625" customWidth="1"/>
-    <col min="3" max="3" width="39.86328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.86328125" customWidth="1"/>
+    <col min="1" max="1" width="21.1640625" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="37.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="37.33203125" customWidth="1"/>
+    <col min="5" max="5" width="39.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>83</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>85</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+        <v>82</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="D2" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="B2" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="E2" s="4"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E2" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+        <v>92</v>
+      </c>
+      <c r="C3" s="11"/>
+      <c r="D3" s="10" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="D4" s="11"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+        <v>93</v>
+      </c>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="10" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="B5" s="11"/>
-      <c r="C5" t="s">
         <v>94</v>
       </c>
-      <c r="D5" s="11" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="B5" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>95</v>
-      </c>
+        <v>99</v>
+      </c>
+      <c r="C6" s="11"/>
       <c r="D6" s="11" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="D7" s="11"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+        <v>101</v>
+      </c>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>100</v>
+        <v>147</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>148</v>
       </c>
       <c r="D8" s="11" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="B9" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="C9" s="20" t="s">
+      <c r="E9" s="22" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="B10" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="D9" s="11" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A10" s="11" t="s">
+      <c r="C10" s="11"/>
+      <c r="D10" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="B10" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="C10" t="s">
-        <v>109</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E10" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="B11" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="C11" t="s">
-        <v>113</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E11" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="C12" s="21" t="s">
+        <v>118</v>
+      </c>
+      <c r="D12" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="B12" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
       <c r="D13" s="11"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="B14" s="11"/>
-      <c r="C14" s="20"/>
+      <c r="C14" s="11"/>
       <c r="D14" s="11"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E14" s="22"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
-        <v>25</v>
+        <v>143</v>
       </c>
       <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
       <c r="D15" s="11"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
-        <v>119</v>
+        <v>144</v>
       </c>
       <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
       <c r="D16" s="11"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="B17" s="11"/>
-      <c r="D17" s="11"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A18" s="11" t="s">
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="E19" t="s">
         <v>121</v>
       </c>
-      <c r="B18" s="11"/>
-      <c r="D18" s="11"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A19" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="C19" t="s">
-        <v>123</v>
-      </c>
-      <c r="D19" s="11"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A20" s="11"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="11" t="s">
+        <v>45</v>
+      </c>
       <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
       <c r="D20" s="11"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A21" s="11"/>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" s="11" t="s">
+        <v>139</v>
+      </c>
       <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
       <c r="D21" s="11"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A22" s="11"/>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" s="11" t="s">
+        <v>140</v>
+      </c>
       <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
       <c r="D22" s="11"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A23" s="11"/>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" s="11" t="s">
+        <v>141</v>
+      </c>
       <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
       <c r="D23" s="11"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A24" s="11"/>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" s="11" t="s">
+        <v>129</v>
+      </c>
       <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
       <c r="D24" s="11"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="11"/>
       <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
       <c r="D25" s="11"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="11"/>
       <c r="B26" s="11"/>
+      <c r="C26" s="11"/>
       <c r="D26" s="11"/>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="11"/>
       <c r="B27" s="11"/>
+      <c r="C27" s="11"/>
       <c r="D27" s="11"/>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" s="11"/>
       <c r="B28" s="11"/>
+      <c r="C28" s="11"/>
       <c r="D28" s="11"/>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" s="11"/>
       <c r="B29" s="11"/>
+      <c r="C29" s="11"/>
       <c r="D29" s="11"/>
     </row>
   </sheetData>

</xml_diff>